<commit_message>
hice tabla 1 depresion 2009
</commit_message>
<xml_diff>
--- a/output/tables/Depresion/tabla1_depresion_2003.xlsx
+++ b/output/tables/Depresion/tabla1_depresion_2003.xlsx
@@ -372,12 +372,12 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>**With symptoms (N=2119)**</t>
+          <t>**Without symptoms (N=2119)**</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>**Con symptoms (N=510)**</t>
+          <t>**With symptoms (N=510)**</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">

</xml_diff>